<commit_message>
feat: SessionStart hook for auto-orchestration of price-tracker and tax agents
Adds a session check hook that detects stale prices (>24h) and upcoming tax
deadlines (90-day window to April 15), then triggers the appropriate agents
in parallel. Also includes live price updates from price-tracker run
(stocks, crypto, Anthropic Series G $40→$50) and 8 new momentum/valuation
signals.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/crypto.xlsx
+++ b/data/crypto.xlsx
@@ -398,20 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L3"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="50.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="22.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -468,7 +454,7 @@
         <v>42000</v>
       </c>
       <c r="F2">
-        <v>97500</v>
+        <v>66927.65</v>
       </c>
       <c r="G2" t="str">
         <v>Small BTC position. Bought during 2022 bear market. Digital gold thesis.</v>
@@ -486,7 +472,7 @@
         <v>2022-12-01</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-02-12</v>
+        <v>2026-02-13</v>
       </c>
     </row>
     <row r="3">
@@ -506,7 +492,7 @@
         <v>2200</v>
       </c>
       <c r="F3">
-        <v>3180</v>
+        <v>1957.72</v>
       </c>
       <c r="G3" t="str">
         <v>Layer 1 ecosystem. Intellectual interest. Not a "crypto person."</v>
@@ -524,7 +510,7 @@
         <v>2023-02-10</v>
       </c>
       <c r="L3" t="str">
-        <v>2026-02-12</v>
+        <v>2026-02-13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>